<commit_message>
Require daily China Sugar News output
</commit_message>
<xml_diff>
--- a/reports/2026/07/Sugar News 2026-07-25.xlsx
+++ b/reports/2026/07/Sugar News 2026-07-25.xlsx
@@ -481,7 +481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col width="55" customWidth="1" style="2" min="2" max="2"/>
@@ -522,6 +522,74 @@
         </is>
       </c>
     </row>
+    <row r="3" ht="116.95" customHeight="1" s="2">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>中国</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>2015—2025年，中国进口甘蔗由105.41万吨增加至359.07万吨，十年增长约240.6%；2026年1—6月累计进口326.12万吨，已相当于2025年全年的90.8%。进口甘蔗持续补充国内糖料供应并提高边境糖厂原料保障，对国内糖价形成利空影响。来源：云糖网（https://www.yntw.com/date/2026/07）</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>利空：进口甘蔗增长补充国内糖料供应并增强边境糖厂原料保障，增加食糖供应预期。</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="123.55" customHeight="1" s="2">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>中国</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>国内食糖工业库存约449万吨，仍处于历史同期偏高水平；6月进口食糖28万吨，市场预计7月以后进口量继续增加。高库存叠加进口到港增长，将继续压制国内现货及郑糖价格的反弹空间。来源：紫金天风期货（https://finance.sina.com.cn/money/future/fmnews/2026-07-23/doc-iniiusky8326649.shtml）</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>利空：高库存与进口到港增加共同扩大可供应量，压制国内现货及郑糖价格。</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="114.2" customHeight="1" s="2">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>中国</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>7月23日夜间起，云南文山、红河、玉溪、普洱等甘蔗产区预报中到大雨、局部暴雨至大暴雨，部分地区伴有短时强降水、大风和冰雹。强降雨可能造成局部农田积水、甘蔗倒伏及田间管理困难，短期不利于甘蔗生长和后续供应。来源：云南网（https://yn.yunnan.cn/system/2026/07/24/034094070.shtml）</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>利多：暴雨、大风和冰雹可能导致积水、倒伏及田间管理困难，使未来糖料供应下降或稳定性减弱。</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="116.95" customHeight="1" s="2">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>中国</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>广西制糖集团报价维持5170—5270元/吨，云南制糖集团报价4980—5030元/吨、部分下调10元/吨，加工糖报价总体稳定。现货需求没有明显改善，国内市场缺少新的上涨驱动，短期糖价预计维持低位震荡。来源：光大期货市场观点（https://goodsfu.10jqka.com.cn/20260723/c678373891.shtml）</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>利空：现货需求偏弱且云南报价下调，国内糖价短期缺少上行动力。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>